<commit_message>
Initial Inverse Kinematics Implementation + restructuring
</commit_message>
<xml_diff>
--- a/parolIKV2.xlsx
+++ b/parolIKV2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fudayl/git/my_robot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8207410-E547-CD40-B522-7DCC0D228C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2277034F-827F-954F-9FA4-250ED2705521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34400" windowHeight="26620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34400" yWindow="600" windowWidth="34400" windowHeight="28200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="L6" s="11" cm="1">
         <f t="array" ref="L6">D16</f>
-        <v>1.5707963267948966</v>
+        <v>0</v>
       </c>
       <c r="M6" s="11">
         <v>176.35</v>
@@ -2380,7 +2380,7 @@
       <c r="AA6" s="13"/>
       <c r="AB6" s="12" cm="1">
         <f t="array" ref="AB6">D16</f>
-        <v>1.5707963267948966</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="12">
         <v>-176.35</v>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="L7" s="11" cm="1">
         <f t="array" ref="L7">D17</f>
-        <v>-1.1170107212763709</v>
+        <v>0</v>
       </c>
       <c r="M7" s="11">
         <v>0</v>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="AB7" s="12" cm="1">
         <f t="array" ref="AB7">D17</f>
-        <v>-1.1170107212763709</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="12">
         <v>0</v>
@@ -3025,11 +3025,11 @@
         <v>30</v>
       </c>
       <c r="C16" s="20">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D16" s="21" cm="1">
         <f t="array" ref="D16">RADIANS(C16)</f>
-        <v>1.5707963267948966</v>
+        <v>0</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
@@ -3117,11 +3117,11 @@
         <v>32</v>
       </c>
       <c r="C17" s="20">
-        <v>-64</v>
+        <v>0</v>
       </c>
       <c r="D17" s="21" cm="1">
         <f t="array" ref="D17">RADIANS(C17)</f>
-        <v>-1.1170107212763709</v>
+        <v>0</v>
       </c>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
@@ -3425,11 +3425,11 @@
       </c>
       <c r="C21" s="28" cm="1">
         <f t="array" ref="C21">R47</f>
-        <v>-89.879404629916664</v>
+        <v>2.6857440500091989E-14</v>
       </c>
       <c r="D21" s="28" cm="1">
         <f t="array" ref="D21">AH41</f>
-        <v>279.07283040314246</v>
+        <v>334.38156826091523</v>
       </c>
       <c r="E21" s="28" cm="1">
         <f t="array" ref="E21">IF(ABS(C21-D21)&lt;0.1,1,0)</f>
@@ -3506,11 +3506,11 @@
       </c>
       <c r="C22" s="28" cm="1">
         <f t="array" ref="C22">R48</f>
-        <v>292.36935804260526</v>
+        <v>282.61675727917168</v>
       </c>
       <c r="D22" s="28" cm="1">
         <f t="array" ref="D22">AH42</f>
-        <v>-89.879404629916721</v>
+        <v>-2.7459575503791794E-14</v>
       </c>
       <c r="E22" s="28" cm="1">
         <f t="array" ref="E22">IF(ABS(C22-D22)&lt;0.1,1,0)</f>
@@ -3580,11 +3580,11 @@
       </c>
       <c r="C23" s="28" cm="1">
         <f t="array" ref="C23">R49</f>
-        <v>279.07240479172719</v>
+        <v>334.38204650037716</v>
       </c>
       <c r="D23" s="28" cm="1">
         <f t="array" ref="D23">AH43</f>
-        <v>292.34856695806133</v>
+        <v>282.59084159964209</v>
       </c>
       <c r="E23" s="28" cm="1">
         <f t="array" ref="E23">IF(ABS(C23-D23)&lt;0.1,1,0)</f>
@@ -3660,11 +3660,11 @@
       </c>
       <c r="C24" s="28" cm="1">
         <f t="array" ref="C24">DEGREES(C27)</f>
-        <v>-63.999999999999986</v>
+        <v>10.000018723968342</v>
       </c>
       <c r="D24" s="28" cm="1">
         <f t="array" ref="D24">DEGREES(D27)</f>
-        <v>26.347179045797283</v>
+        <v>-3.0555237504089516E-2</v>
       </c>
       <c r="E24" s="8"/>
       <c r="G24" s="8"/>
@@ -3730,11 +3730,11 @@
       </c>
       <c r="C25" s="28" cm="1">
         <f t="array" ref="C25">DEGREES(C28)</f>
-        <v>-10.00001872396834</v>
+        <v>6.3541887885436076E-15</v>
       </c>
       <c r="D25" s="28" cm="1">
         <f t="array" ref="D25">DEGREES(D28)</f>
-        <v>8.9785681500312382</v>
+        <v>-79.994671222381413</v>
       </c>
       <c r="E25" s="8"/>
       <c r="G25" s="6"/>
@@ -3827,11 +3827,11 @@
       </c>
       <c r="C26" s="28" cm="1">
         <f t="array" ref="C26">DEGREES(C29)</f>
-        <v>90</v>
+        <v>7.5726298296413201E-15</v>
       </c>
       <c r="D26" s="28" cm="1">
         <f t="array" ref="D26">DEGREES(D29)</f>
-        <v>-9.0049402725160377</v>
+        <v>90.005308659651874</v>
       </c>
       <c r="E26" s="8"/>
       <c r="G26" s="6"/>
@@ -3921,11 +3921,11 @@
       </c>
       <c r="C27" s="28">
         <f>ATAN2(Q49,P49)</f>
-        <v>-1.1170107212763707</v>
+        <v>0.17453325199432956</v>
       </c>
       <c r="D27" s="28" cm="1">
         <f t="array" ref="D27">ATAN2(AE41/COS(D28),AE42/COS(D28))</f>
-        <v>0.45984502296162044</v>
+        <v>-5.3328949817521641E-4</v>
       </c>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
@@ -3999,11 +3999,11 @@
       </c>
       <c r="C28" s="28">
         <f>ATAN2((P49^2+Q49^2)^0.5,-O49)</f>
-        <v>-0.17453325199432954</v>
+        <v>1.109015156533957E-16</v>
       </c>
       <c r="D28" s="28" cm="1">
         <f t="array" ref="D28">ATAN2((AF43^2+AG43^2)^0.5,-AE43)</f>
-        <v>0.15670557633274132</v>
+        <v>-1.3961703968809127</v>
       </c>
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
@@ -4070,11 +4070,11 @@
       </c>
       <c r="C29" s="28">
         <f>ATAN2(O47,O48)</f>
-        <v>1.5707963267948966</v>
+        <v>1.3216732356197833E-16</v>
       </c>
       <c r="D29" s="28" cm="1">
         <f t="array" ref="D29">ATAN2(AF43/COS(D28),AE43/COS(D28))</f>
-        <v>-0.1571658567008403</v>
+        <v>1.5708889803846895</v>
       </c>
       <c r="E29" s="8"/>
       <c r="G29" s="8"/>
@@ -4089,10 +4089,10 @@
       </c>
       <c r="O29" s="12" cm="1">
         <f t="array" ref="O29:R32">MMULT(_xlfn.ANCHORARRAY(O23),I31:L34)</f>
+        <v>-4.9669175696028064E-17</v>
+      </c>
+      <c r="P29" s="12">
         <v>-1</v>
-      </c>
-      <c r="P29" s="12">
-        <v>-1.1563164261339596E-17</v>
       </c>
       <c r="Q29" s="12">
         <v>1.3216732356197833E-16</v>
@@ -4116,13 +4116,13 @@
       </c>
       <c r="AE29" s="12" cm="1">
         <f t="array" ref="AE29:AH32">MMULT(_xlfn.ANCHORARRAY(AE23),Y31:AB34)</f>
-        <v>-7.0941556198671339E-17</v>
+        <v>-0.17373974471989401</v>
       </c>
       <c r="AF29" s="12">
         <v>0.98479160288086642</v>
       </c>
       <c r="AG29" s="12">
-        <v>0.17373974471989395</v>
+        <v>-1.2060415930063873E-16</v>
       </c>
       <c r="AH29" s="12">
         <v>235.90240797282857</v>
@@ -4154,10 +4154,10 @@
       <c r="M30" s="6"/>
       <c r="N30" s="33"/>
       <c r="O30" s="12">
-        <v>-1.1563164261339602E-17</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="P30" s="12">
-        <v>-0.98480769626481723</v>
+        <v>-7.1865243911658964E-17</v>
       </c>
       <c r="Q30" s="12">
         <v>-0.1736484994970689</v>
@@ -4178,13 +4178,13 @@
       <c r="AC30" s="6"/>
       <c r="AD30" s="33"/>
       <c r="AE30" s="12">
+        <v>6.0312441006962954E-17</v>
+      </c>
+      <c r="AF30" s="12">
+        <v>-1.1182618827627998E-16</v>
+      </c>
+      <c r="AG30" s="12">
         <v>-1</v>
-      </c>
-      <c r="AF30" s="12">
-        <v>-5.0593848318912331E-17</v>
-      </c>
-      <c r="AG30" s="12">
-        <v>-1.2154478096433061E-16</v>
       </c>
       <c r="AH30" s="12">
         <v>-2.2400190671900561E-14</v>
@@ -4213,11 +4213,11 @@
       </c>
       <c r="I31" s="12" cm="1">
         <f t="array" ref="I31">COS(L6)</f>
-        <v>6.123233995736766E-17</v>
+        <v>1</v>
       </c>
       <c r="J31" s="12" cm="1">
         <f t="array" ref="J31">-SIN(L6)</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K31" s="12">
         <v>0</v>
@@ -4229,10 +4229,10 @@
       <c r="M31" s="22"/>
       <c r="N31" s="33"/>
       <c r="O31" s="12">
-        <v>1.3216732356197833E-16</v>
+        <v>0.1736484994970689</v>
       </c>
       <c r="P31" s="12">
-        <v>-0.1736484994970689</v>
+        <v>1.2153441960768702E-16</v>
       </c>
       <c r="Q31" s="12">
         <v>0.98480769626481723</v>
@@ -4250,15 +4250,15 @@
       </c>
       <c r="Y31" s="12" cm="1">
         <f t="array" ref="Y31">COS(AB6)</f>
-        <v>6.123233995736766E-17</v>
+        <v>1</v>
       </c>
       <c r="Z31" s="12" cm="1">
         <f t="array" ref="Z31">-SIN(AB6)*COS(Z6)</f>
-        <v>-6.123233995736766E-17</v>
+        <v>0</v>
       </c>
       <c r="AA31" s="12" cm="1">
         <f t="array" ref="AA31">SIN(AB6)*SIN(Z6)</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AB31" s="12" cm="1">
         <f t="array" ref="AB31">AA6*COS(AB6)</f>
@@ -4267,13 +4267,13 @@
       <c r="AC31" s="22"/>
       <c r="AD31" s="33"/>
       <c r="AE31" s="12">
-        <v>-1.1090611737634209E-16</v>
+        <v>-0.98479160288086642</v>
       </c>
       <c r="AF31" s="12">
-        <v>-0.17373974471989395</v>
+        <v>-0.17373974471989401</v>
       </c>
       <c r="AG31" s="12">
-        <v>0.98479160288086642</v>
+        <v>-3.9966532048785048E-17</v>
       </c>
       <c r="AH31" s="12">
         <v>299.9648160716315</v>
@@ -4301,11 +4301,11 @@
       <c r="H32" s="36"/>
       <c r="I32" s="12" cm="1">
         <f t="array" ref="I32">SIN(L6)*COS(J6)</f>
-        <v>6.123233995736766E-17</v>
+        <v>0</v>
       </c>
       <c r="J32" s="12" cm="1">
         <f t="array" ref="J32">COS(L6)*COS(J6)</f>
-        <v>3.749399456654644E-33</v>
+        <v>6.123233995736766E-17</v>
       </c>
       <c r="K32" s="12" cm="1">
         <f t="array" ref="K32">-SIN(J6)</f>
@@ -4337,15 +4337,15 @@
       <c r="X32" s="36"/>
       <c r="Y32" s="12" cm="1">
         <f t="array" ref="Y32">SIN(AB6)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z32" s="12" cm="1">
         <f t="array" ref="Z32">COS(AB6)*COS(Z6)</f>
-        <v>3.749399456654644E-33</v>
+        <v>6.123233995736766E-17</v>
       </c>
       <c r="AA32" s="12" cm="1">
         <f t="array" ref="AA32">-COS(AB6)*SIN(Z6)</f>
-        <v>6.123233995736766E-17</v>
+        <v>1</v>
       </c>
       <c r="AB32" s="12" cm="1">
         <f t="array" ref="AB32">AA6*SIN(AB6)</f>
@@ -4388,11 +4388,11 @@
       <c r="H33" s="36"/>
       <c r="I33" s="12" cm="1">
         <f t="array" ref="I33">SIN(L6)*SIN(J6)</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J33" s="12" cm="1">
         <f t="array" ref="J33">COS(L6)*SIN(J6)</f>
-        <v>-6.123233995736766E-17</v>
+        <v>-1</v>
       </c>
       <c r="K33" s="12" cm="1">
         <f t="array" ref="K33">COS(J6)</f>
@@ -4529,13 +4529,13 @@
       </c>
       <c r="O35" s="12" cm="1">
         <f t="array" ref="O35:R38">MMULT(_xlfn.ANCHORARRAY(O29),I37:L40)</f>
-        <v>-0.43837114678907757</v>
+        <v>-4.9669175696028064E-17</v>
       </c>
       <c r="P35" s="12">
-        <v>-0.89879404629916682</v>
+        <v>7.0934983604610671E-17</v>
       </c>
       <c r="Q35" s="12">
-        <v>1.1563164261339604E-17</v>
+        <v>1</v>
       </c>
       <c r="R35" s="12">
         <v>1.3640708143894156E-14</v>
@@ -4556,13 +4556,13 @@
       </c>
       <c r="AE35" s="12" cm="1">
         <f t="array" ref="AE35:AH38">MMULT(_xlfn.ANCHORARRAY(AE29),Y37:AB40)</f>
-        <v>-0.88512482951473626</v>
+        <v>-0.17373974471989401</v>
       </c>
       <c r="AF35" s="12">
-        <v>0.17373974471989398</v>
+        <v>-6.0303065085876511E-17</v>
       </c>
       <c r="AG35" s="12">
-        <v>-0.43170422430313909</v>
+        <v>-0.98479160288086642</v>
       </c>
       <c r="AH35" s="12">
         <v>235.90240797282857</v>
@@ -4595,13 +4595,13 @@
       <c r="M36" s="6"/>
       <c r="N36" s="33"/>
       <c r="O36" s="12">
-        <v>0.15607423749674945</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="P36" s="12">
-        <v>-7.6122491862732677E-2</v>
+        <v>-0.1736484994970689</v>
       </c>
       <c r="Q36" s="12">
-        <v>0.98480769626481723</v>
+        <v>6.1232339957367648E-17</v>
       </c>
       <c r="R36" s="12">
         <v>299.98160722887854</v>
@@ -4619,13 +4619,13 @@
       <c r="AC36" s="6"/>
       <c r="AD36" s="33"/>
       <c r="AE36" s="12">
-        <v>-0.4383711467890774</v>
+        <v>6.0312441006962954E-17</v>
       </c>
       <c r="AF36" s="12">
-        <v>-1.7658004355897925E-16</v>
+        <v>-1</v>
       </c>
       <c r="AG36" s="12">
-        <v>0.89879404629916693</v>
+        <v>5.0593848318912324E-17</v>
       </c>
       <c r="AH36" s="12">
         <v>-2.2400190671900561E-14</v>
@@ -4655,11 +4655,11 @@
       </c>
       <c r="I37" s="12" cm="1">
         <f t="array" ref="I37">COS(L7)</f>
-        <v>0.43837114678907746</v>
+        <v>1</v>
       </c>
       <c r="J37" s="12" cm="1">
         <f t="array" ref="J37">-SIN(L7)</f>
-        <v>0.89879404629916693</v>
+        <v>0</v>
       </c>
       <c r="K37" s="12">
         <v>0</v>
@@ -4671,13 +4671,13 @@
       <c r="M37" s="22"/>
       <c r="N37" s="33"/>
       <c r="O37" s="12">
-        <v>-0.88513929415241599</v>
+        <v>0.1736484994970689</v>
       </c>
       <c r="P37" s="12">
-        <v>0.43171127917831753</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="Q37" s="12">
-        <v>0.17364849949706895</v>
+        <v>-6.1232339957367648E-17</v>
       </c>
       <c r="R37" s="12">
         <v>235.90127687389543</v>
@@ -4692,15 +4692,15 @@
       </c>
       <c r="Y37" s="12" cm="1">
         <f t="array" ref="Y37">COS(AB7)</f>
-        <v>0.43837114678907746</v>
+        <v>1</v>
       </c>
       <c r="Z37" s="12" cm="1">
         <f t="array" ref="Z37">-SIN(AB7)*COS(Z7)</f>
-        <v>5.503526259464864E-17</v>
+        <v>0</v>
       </c>
       <c r="AA37" s="12" cm="1">
         <f t="array" ref="AA37">SIN(AB7)*SIN(Z7)</f>
-        <v>-0.89879404629916693</v>
+        <v>0</v>
       </c>
       <c r="AB37" s="12" cm="1">
         <f t="array" ref="AB37">AA7*COS(AB7)</f>
@@ -4709,13 +4709,13 @@
       <c r="AC37" s="22"/>
       <c r="AD37" s="33"/>
       <c r="AE37" s="12">
-        <v>0.15615624815977774</v>
+        <v>-0.98479160288086642</v>
       </c>
       <c r="AF37" s="12">
-        <v>0.98479160288086642</v>
+        <v>-5.0605023161579869E-17</v>
       </c>
       <c r="AG37" s="12">
-        <v>7.6162491135701629E-2</v>
+        <v>0.17373974471989401</v>
       </c>
       <c r="AH37" s="12">
         <v>299.9648160716315</v>
@@ -4743,11 +4743,11 @@
       <c r="H38" s="36"/>
       <c r="I38" s="12" cm="1">
         <f t="array" ref="I38">SIN(L7)*COS(J7)</f>
-        <v>-5.503526259464864E-17</v>
+        <v>0</v>
       </c>
       <c r="J38" s="12" cm="1">
         <f t="array" ref="J38">COS(L7)*COS(J7)</f>
-        <v>2.6842491087689912E-17</v>
+        <v>6.123233995736766E-17</v>
       </c>
       <c r="K38" s="12" cm="1">
         <f t="array" ref="K38">-SIN(J7)</f>
@@ -4779,15 +4779,15 @@
       <c r="X38" s="36"/>
       <c r="Y38" s="12" cm="1">
         <f t="array" ref="Y38">SIN(AB7)</f>
-        <v>-0.89879404629916693</v>
+        <v>0</v>
       </c>
       <c r="Z38" s="12" cm="1">
         <f t="array" ref="Z38">COS(AB7)*COS(Z7)</f>
-        <v>2.6842491087689912E-17</v>
+        <v>6.123233995736766E-17</v>
       </c>
       <c r="AA38" s="12" cm="1">
         <f t="array" ref="AA38">-COS(AB7)*SIN(Z7)</f>
-        <v>-0.43837114678907746</v>
+        <v>-1</v>
       </c>
       <c r="AB38" s="12" cm="1">
         <f t="array" ref="AB38">AA7*SIN(AB7)</f>
@@ -4830,11 +4830,11 @@
       <c r="H39" s="36"/>
       <c r="I39" s="12" cm="1">
         <f t="array" ref="I39">SIN(L7)*SIN(J7)</f>
-        <v>-0.89879404629916693</v>
+        <v>0</v>
       </c>
       <c r="J39" s="12" cm="1">
         <f t="array" ref="J39">COS(L7)*SIN(J7)</f>
-        <v>0.43837114678907746</v>
+        <v>1</v>
       </c>
       <c r="K39" s="12" cm="1">
         <f t="array" ref="K39">COS(J7)</f>
@@ -4971,13 +4971,13 @@
       </c>
       <c r="O41" s="12" cm="1">
         <f t="array" ref="O41:R44">MMULT(_xlfn.ANCHORARRAY(O35),I43:L46)</f>
-        <v>-0.43837114678907757</v>
+        <v>-4.9669175696028064E-17</v>
       </c>
       <c r="P41" s="12">
-        <v>-6.6598426855988242E-17</v>
+        <v>-1</v>
       </c>
       <c r="Q41" s="12">
-        <v>-0.89879404629916682</v>
+        <v>1.3216732356197833E-16</v>
       </c>
       <c r="R41" s="12">
         <v>1.3640708143894156E-14</v>
@@ -4998,16 +4998,16 @@
       </c>
       <c r="AE41" s="12" cm="1">
         <f t="array" ref="AE41:AH44">MMULT(_xlfn.ANCHORARRAY(AE35),Y43:AB46)</f>
-        <v>0.88514092332649108</v>
+        <v>0.1737397439741433</v>
       </c>
       <c r="AF41" s="12">
-        <v>0.17365773398139103</v>
+        <v>-1.6097611015176289E-5</v>
       </c>
       <c r="AG41" s="12">
-        <v>0.43170422430313909</v>
+        <v>0.98479160288086642</v>
       </c>
       <c r="AH41" s="12">
-        <v>279.07283040314246</v>
+        <v>334.38156826091523</v>
       </c>
       <c r="AI41" s="7"/>
       <c r="AJ41" s="8"/>
@@ -5037,13 +5037,13 @@
       <c r="M42" s="6"/>
       <c r="N42" s="33"/>
       <c r="O42" s="12">
-        <v>0.15607423749674945</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="P42" s="12">
-        <v>-0.98480769626481723</v>
+        <v>-7.1865243911658964E-17</v>
       </c>
       <c r="Q42" s="12">
-        <v>-7.6122491862732622E-2</v>
+        <v>-0.1736484994970689</v>
       </c>
       <c r="R42" s="12">
         <v>299.98160722887854</v>
@@ -5061,16 +5061,16 @@
       <c r="AC42" s="6"/>
       <c r="AD42" s="33"/>
       <c r="AE42" s="12">
-        <v>0.43837114490743773</v>
+        <v>-9.2653589660550567E-5</v>
       </c>
       <c r="AF42" s="12">
-        <v>-4.0616660353660227E-5</v>
+        <v>-0.99999999570765619</v>
       </c>
       <c r="AG42" s="12">
-        <v>-0.89879404629916693</v>
+        <v>-1.7305852770798714E-16</v>
       </c>
       <c r="AH42" s="12">
-        <v>-89.879404629916721</v>
+        <v>-2.7459575503791794E-14</v>
       </c>
       <c r="AI42" s="7"/>
       <c r="AJ42" s="8"/>
@@ -5113,13 +5113,13 @@
       <c r="M43" s="22"/>
       <c r="N43" s="33"/>
       <c r="O43" s="12">
-        <v>-0.88513929415241599</v>
+        <v>0.1736484994970689</v>
       </c>
       <c r="P43" s="12">
-        <v>-0.17364849949706893</v>
+        <v>1.2153441960768702E-16</v>
       </c>
       <c r="Q43" s="12">
-        <v>0.43171127917831753</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="R43" s="12">
         <v>235.90127687389543</v>
@@ -5151,16 +5151,16 @@
       <c r="AC43" s="22"/>
       <c r="AD43" s="33"/>
       <c r="AE43" s="12">
-        <v>-0.15606500301242701</v>
+        <v>0.98479159865380228</v>
       </c>
       <c r="AF43" s="12">
-        <v>0.98480606709074214</v>
+        <v>-9.1244477074449602E-5</v>
       </c>
       <c r="AG43" s="12">
-        <v>-7.6162491135701504E-2</v>
+        <v>-0.17373974471989401</v>
       </c>
       <c r="AH43" s="12">
-        <v>292.34856695806133</v>
+        <v>282.59084159964209</v>
       </c>
       <c r="AI43" s="7"/>
       <c r="AJ43" s="8"/>
@@ -5413,16 +5413,16 @@
       </c>
       <c r="O47" s="12" cm="1">
         <f t="array" ref="O47:R50">MMULT(_xlfn.ANCHORARRAY(O41),I49:L52)</f>
-        <v>3.9755935768298324E-17</v>
+        <v>1</v>
       </c>
       <c r="P47" s="12">
-        <v>-0.43837114678907757</v>
+        <v>-1.1090151565339572E-16</v>
       </c>
       <c r="Q47" s="12">
-        <v>-0.89879404629916682</v>
+        <v>1.3216732356197833E-16</v>
       </c>
       <c r="R47" s="12">
-        <v>-89.879404629916664</v>
+        <v>2.6857440500091989E-14</v>
       </c>
       <c r="S47" s="7"/>
       <c r="T47" s="8"/>
@@ -5468,16 +5468,16 @@
       <c r="M48" s="6"/>
       <c r="N48" s="33"/>
       <c r="O48" s="12">
+        <v>1.3216732356197833E-16</v>
+      </c>
+      <c r="P48" s="12">
         <v>0.98480769626481723</v>
       </c>
-      <c r="P48" s="12">
-        <v>0.1560742374967494</v>
-      </c>
       <c r="Q48" s="12">
-        <v>-7.6122491862732622E-2</v>
+        <v>-0.1736484994970689</v>
       </c>
       <c r="R48" s="12">
-        <v>292.36935804260526</v>
+        <v>282.61675727917168</v>
       </c>
       <c r="S48" s="7"/>
       <c r="T48" s="8"/>
@@ -5536,16 +5536,16 @@
       <c r="M49" s="22"/>
       <c r="N49" s="33"/>
       <c r="O49" s="12">
-        <v>0.17364849949706887</v>
+        <v>-1.109015156533957E-16</v>
       </c>
       <c r="P49" s="12">
-        <v>-0.88513929415241599</v>
+        <v>0.1736484994970689</v>
       </c>
       <c r="Q49" s="12">
-        <v>0.43171127917831753</v>
+        <v>0.98480769626481723</v>
       </c>
       <c r="R49" s="12">
-        <v>279.07240479172719</v>
+        <v>334.38204650037716</v>
       </c>
       <c r="S49" s="7"/>
       <c r="T49" s="8"/>

</xml_diff>